<commit_message>
fix(v4): bump GNSS ECO board revision to V4.1
</commit_message>
<xml_diff>
--- a/hardware/expansion-board-v4/CHECKLIST.xlsx
+++ b/hardware/expansion-board-v4/CHECKLIST.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="V4.0 核对清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="V4.1 核对清单" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'V4.0 核对清单'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'V4.1 核对清单'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>